<commit_message>
refine: clarify Excel import and show cut total
</commit_message>
<xml_diff>
--- a/public/templates/cut-master-pro-input-template.xlsx
+++ b/public/templates/cut-master-pro-input-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_入力" sheetId="1" r:id="R310895f009cf4d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_入力例" sheetId="2" r:id="Re67dcf8c313a42e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_使い方" sheetId="3" r:id="Ra300cc21c8dc41c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_入力" sheetId="1" r:id="Rca739c7f6a374f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_入力例" sheetId="2" r:id="Rc8ff2d2c3a1c44a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_使い方" sheetId="3" r:id="R78d7ecc9394048b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3273,7 +3273,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="42" t="str">
-        <x:v>アプリの「部材リスト取込」で保存したExcelを選ぶ</x:v>
+        <x:v>アプリの「Excelから寸法取込」で保存したExcelを選ぶ</x:v>
       </x:c>
       <x:c r="C10" s="42"/>
       <x:c r="D10" s="42"/>
@@ -3283,7 +3283,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="42" t="str">
-        <x:v>取込内容を確認し「部材一覧を置き換える」を押す</x:v>
+        <x:v>取込内容を確認し「切断寸法を置き換える」を押す</x:v>
       </x:c>
       <x:c r="C11" s="42"/>
       <x:c r="D11" s="42"/>

</xml_diff>

<commit_message>
fix: clarify Excel import template
</commit_message>
<xml_diff>
--- a/public/templates/cut-master-pro-input-template.xlsx
+++ b/public/templates/cut-master-pro-input-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_入力" sheetId="1" r:id="Rca739c7f6a374f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_入力例" sheetId="2" r:id="Rc8ff2d2c3a1c44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_使い方" sheetId="3" r:id="R78d7ecc9394048b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_入力" sheetId="1" r:id="Rdaf9c5db1e3c471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_入力例" sheetId="2" r:id="Re69af875eb3e4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_使い方" sheetId="3" r:id="R4b0b8a51c6044fbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -241,7 +241,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -350,6 +350,24 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -3145,25 +3163,27 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="23" t="str">
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="59" t="str">
+        <x:v>配管はパイプ番号、製作品は部材名を入力します。
+両方を入れても構いません。</x:v>
+      </x:c>
+      <x:c r="B7" s="60" t="str">
         <x:v>配管はパイプ番号、製作品は部材名を入力します。両方を入れても構いません。</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="str">
+      <x:c r="C7" s="61" t="str">
         <x:v>配管はパイプ番号、製作品は部材名を入力します。両方を入れても構いません。</x:v>
       </x:c>
-      <x:c r="C7" s="25" t="str">
-        <x:v>配管はパイプ番号、製作品は部材名を入力します。両方を入れても構いません。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="30" t="str">
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="62" t="str">
+        <x:v>本数を空欄にすると1本として取り込みます。
+パイプ番号・部材名も空欄にできます。</x:v>
+      </x:c>
+      <x:c r="B9" s="63" t="str">
         <x:v>本数を空欄にすると1本として取り込みます。パイプ番号・部材名も空欄にできます。</x:v>
       </x:c>
-      <x:c r="B9" s="31" t="str">
-        <x:v>本数を空欄にすると1本として取り込みます。パイプ番号・部材名も空欄にできます。</x:v>
-      </x:c>
-      <x:c r="C9" s="32" t="str">
+      <x:c r="C9" s="64" t="str">
         <x:v>本数を空欄にすると1本として取り込みます。パイプ番号・部材名も空欄にできます。</x:v>
       </x:c>
     </x:row>

</xml_diff>